<commit_message>
Quellen und Testdaten final überprüft
</commit_message>
<xml_diff>
--- a/Testdaten/Testdaten von und für GPT-4o/OpenCart-Testfälle GPT-4o_ausgewertet.xlsx
+++ b/Testdaten/Testdaten von und für GPT-4o/OpenCart-Testfälle GPT-4o_ausgewertet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Marvi\Desktop\Bachelor-Thesis\Testdaten\Testdaten von und für GPT-4o\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6966BB80-FF24-4594-BBE8-EB7FC6AF18C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0322790-B4CA-43E2-B1DD-91A1B59F984B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="3" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Szenarien" sheetId="33" r:id="rId1"/>
@@ -6341,7 +6341,7 @@
         <v>15</v>
       </c>
       <c r="H12" s="4" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="I12" s="4">
         <v>1</v>

</xml_diff>